<commit_message>
tune milk cow durations and add save inspection tooling
</commit_message>
<xml_diff>
--- a/Data Sheets/Sandbox.xlsx
+++ b/Data Sheets/Sandbox.xlsx
@@ -469,6 +469,9 @@
     <t>Milk Cow I</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>Spawn Milk Cow</t>
   </si>
   <si>
@@ -593,9 +596,6 @@
   </si>
   <si>
     <t>Build La Rochelle Submarine Pen 1</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t>InstallEquipment</t>
@@ -43012,8 +43012,8 @@
       <c r="B52" s="12">
         <v>14397</v>
       </c>
-      <c r="C52" s="13">
-        <v>12</v>
+      <c r="C52" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D52" s="13">
         <v>0</v>
@@ -43025,10 +43025,10 @@
         <v>-44.01786</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J52" s="16" t="s">
         <v>86</v>
@@ -43037,18 +43037,18 @@
       <c r="L52" s="16"/>
       <c r="M52" s="16"/>
       <c r="N52" s="11" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" s="13" customFormat="1">
       <c r="A53" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B53" s="12">
         <v>14458</v>
       </c>
-      <c r="C53" s="13">
-        <v>12</v>
+      <c r="C53" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D53" s="13">
         <v>0</v>
@@ -43060,10 +43060,10 @@
         <v>-44.71251</v>
       </c>
       <c r="G53" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J53" s="16" t="s">
         <v>86</v>
@@ -43072,18 +43072,18 @@
       <c r="L53" s="16"/>
       <c r="M53" s="16"/>
       <c r="N53" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="54" s="13" customFormat="1">
       <c r="A54" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B54" s="12">
         <v>14458</v>
       </c>
-      <c r="C54" s="13">
-        <v>12</v>
+      <c r="C54" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D54" s="13">
         <v>0</v>
@@ -43095,10 +43095,10 @@
         <v>-45.72372</v>
       </c>
       <c r="G54" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J54" s="16" t="s">
         <v>86</v>
@@ -43107,18 +43107,18 @@
       <c r="L54" s="16"/>
       <c r="M54" s="16"/>
       <c r="N54" s="11" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="55" s="13" customFormat="1">
       <c r="A55" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B55" s="12">
         <v>14458</v>
       </c>
-      <c r="C55" s="13">
-        <v>12</v>
+      <c r="C55" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D55" s="13">
         <v>0</v>
@@ -43130,10 +43130,10 @@
         <v>-57.53769</v>
       </c>
       <c r="G55" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J55" s="16" t="s">
         <v>86</v>
@@ -43142,18 +43142,18 @@
       <c r="L55" s="16"/>
       <c r="M55" s="16"/>
       <c r="N55" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="56" s="13" customFormat="1">
       <c r="A56" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B56" s="12">
         <v>14458</v>
       </c>
-      <c r="C56" s="13">
-        <v>12</v>
+      <c r="C56" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D56" s="13">
         <v>0</v>
@@ -43165,10 +43165,10 @@
         <v>-49.73495</v>
       </c>
       <c r="G56" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J56" s="16" t="s">
         <v>86</v>
@@ -43177,18 +43177,18 @@
       <c r="L56" s="16"/>
       <c r="M56" s="16"/>
       <c r="N56" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="57" s="13" customFormat="1">
       <c r="A57" s="11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B57" s="12">
         <v>14458</v>
       </c>
-      <c r="C57" s="13">
-        <v>12</v>
+      <c r="C57" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D57" s="13">
         <v>0</v>
@@ -43200,10 +43200,10 @@
         <v>-46.00481</v>
       </c>
       <c r="G57" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J57" s="16" t="s">
         <v>86</v>
@@ -43212,18 +43212,18 @@
       <c r="L57" s="16"/>
       <c r="M57" s="16"/>
       <c r="N57" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="58" s="13" customFormat="1">
       <c r="A58" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B58" s="12">
         <v>14458</v>
       </c>
-      <c r="C58" s="13">
-        <v>12</v>
+      <c r="C58" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D58" s="13">
         <v>0</v>
@@ -43235,10 +43235,10 @@
         <v>-43.61742</v>
       </c>
       <c r="G58" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J58" s="16" t="s">
         <v>86</v>
@@ -43247,18 +43247,18 @@
       <c r="L58" s="16"/>
       <c r="M58" s="16"/>
       <c r="N58" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="59" s="13" customFormat="1">
       <c r="A59" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B59" s="12">
         <v>14458</v>
       </c>
-      <c r="C59" s="13">
-        <v>12</v>
+      <c r="C59" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D59" s="13">
         <v>0</v>
@@ -43270,10 +43270,10 @@
         <v>-32.59997</v>
       </c>
       <c r="G59" s="13" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J59" s="16" t="s">
         <v>86</v>
@@ -43282,18 +43282,18 @@
       <c r="L59" s="16"/>
       <c r="M59" s="16"/>
       <c r="N59" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="60" s="13" customFormat="1">
       <c r="A60" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B60" s="12">
         <v>14458</v>
       </c>
-      <c r="C60" s="13">
-        <v>12</v>
+      <c r="C60" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D60" s="13">
         <v>0</v>
@@ -43305,10 +43305,10 @@
         <v>-44.66367</v>
       </c>
       <c r="G60" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J60" s="16" t="s">
         <v>86</v>
@@ -43317,18 +43317,18 @@
       <c r="L60" s="16"/>
       <c r="M60" s="16"/>
       <c r="N60" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" s="13" customFormat="1">
       <c r="A61" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B61" s="12">
         <v>14458</v>
       </c>
-      <c r="C61" s="13">
-        <v>12</v>
+      <c r="C61" s="13" t="s">
+        <v>121</v>
       </c>
       <c r="D61" s="13">
         <v>0</v>
@@ -43340,10 +43340,10 @@
         <v>-57.48545</v>
       </c>
       <c r="G61" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J61" s="16" t="s">
         <v>86</v>
@@ -43352,12 +43352,12 @@
       <c r="L61" s="16"/>
       <c r="M61" s="16"/>
       <c r="N61" s="11" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B62" s="8">
         <v>14246</v>
@@ -43375,19 +43375,19 @@
         <v>10000</v>
       </c>
       <c r="I62" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J62" s="7"/>
       <c r="K62" s="7"/>
       <c r="L62" s="7"/>
       <c r="M62" s="7"/>
       <c r="N62" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B63" s="8">
         <v>14246</v>
@@ -43405,19 +43405,19 @@
         <v>10000</v>
       </c>
       <c r="I63" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J63" s="7"/>
       <c r="K63" s="7"/>
       <c r="L63" s="7"/>
       <c r="M63" s="7"/>
       <c r="N63" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B64" s="8">
         <v>14246</v>
@@ -43435,19 +43435,19 @@
         <v>10000</v>
       </c>
       <c r="I64" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J64" s="7"/>
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
       <c r="M64" s="7"/>
       <c r="N64" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B65" s="8">
         <v>14246</v>
@@ -43465,19 +43465,19 @@
         <v>10000</v>
       </c>
       <c r="I65" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J65" s="7"/>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
       <c r="M65" s="7"/>
       <c r="N65" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B66" s="8">
         <v>14246</v>
@@ -43495,19 +43495,19 @@
         <v>10000</v>
       </c>
       <c r="I66" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J66" s="7"/>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
       <c r="M66" s="7"/>
       <c r="N66" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B67" s="8">
         <v>14246</v>
@@ -43525,19 +43525,19 @@
         <v>10000</v>
       </c>
       <c r="I67" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J67" s="7"/>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
       <c r="M67" s="7"/>
       <c r="N67" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B68" s="8">
         <v>14246</v>
@@ -43555,19 +43555,19 @@
         <v>10000</v>
       </c>
       <c r="I68" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J68" s="7"/>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
       <c r="M68" s="7"/>
       <c r="N68" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B69" s="8">
         <v>14246</v>
@@ -43585,19 +43585,19 @@
         <v>10000</v>
       </c>
       <c r="I69" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J69" s="7"/>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
       <c r="M69" s="7"/>
       <c r="N69" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B70" s="8">
         <v>14246</v>
@@ -43615,19 +43615,19 @@
         <v>10000</v>
       </c>
       <c r="I70" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J70" s="7"/>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
       <c r="M70" s="7"/>
       <c r="N70" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B71" s="8">
         <v>14246</v>
@@ -43645,25 +43645,25 @@
         <v>10000</v>
       </c>
       <c r="I71" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J71" s="7"/>
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
       <c r="M71" s="7"/>
       <c r="N71" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="72" ht="15">
       <c r="A72" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B72" s="5">
         <v>14246</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="D72" s="5">
         <v>0</v>
@@ -43702,7 +43702,7 @@
         <v>14246</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="D73" s="5">
         <v>0</v>
@@ -43714,7 +43714,7 @@
         <v>-1.202584</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H73" s="5"/>
       <c r="I73" s="5" t="s">
@@ -43743,7 +43743,7 @@
         <v>14246</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="D74" s="5">
         <v>0</v>
@@ -43780,7 +43780,7 @@
         <v>14772</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="D75" s="5">
         <v>0</v>
@@ -43819,7 +43819,7 @@
         <v>14246</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="D76" s="5">
         <v>0</v>
@@ -43858,7 +43858,7 @@
         <v>14246</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>163</v>
+        <v>121</v>
       </c>
       <c r="D77" s="5">
         <v>0</v>

</xml_diff>